<commit_message>
QLT BAO CAO 01
</commit_message>
<xml_diff>
--- a/Quan Trac Lun/Data/HD XL01/KM0+500.xlsx
+++ b/Quan Trac Lun/Data/HD XL01/KM0+500.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Vba\bketech\Quan Trac Lun\Data\HD XL01\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\VBA Project\bketech\Quan Trac Lun\Data\HD XL01\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EFE44700-1151-4D71-8B54-87C3F5F03114}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68AC9C09-974D-4C34-91CF-B6EE8A5CBC02}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-8325" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{2C402617-1403-418F-9928-C6EF4DD57BF2}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{2C402617-1403-418F-9928-C6EF4DD57BF2}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -245,7 +245,7 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Aptos Narrow"/>
+      <name val="Arial"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -263,14 +263,14 @@
       <b/>
       <sz val="13"/>
       <color theme="1"/>
-      <name val="Aptos Display"/>
+      <name val="Times New Roman"/>
       <family val="1"/>
       <scheme val="major"/>
     </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Aptos Display"/>
+      <name val="Times New Roman"/>
       <family val="1"/>
       <scheme val="major"/>
     </font>
@@ -279,7 +279,7 @@
       <u/>
       <sz val="13"/>
       <color theme="1"/>
-      <name val="Aptos Display"/>
+      <name val="Times New Roman"/>
       <family val="1"/>
       <scheme val="major"/>
     </font>
@@ -287,20 +287,20 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Aptos Display"/>
+      <name val="Times New Roman"/>
       <family val="1"/>
       <scheme val="major"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
-      <name val="Aptos Display"/>
+      <name val="Times New Roman"/>
       <family val="1"/>
       <scheme val="major"/>
     </font>
     <font>
       <sz val="11"/>
-      <name val="Aptos Display"/>
+      <name val="Times New Roman"/>
       <family val="1"/>
       <scheme val="major"/>
     </font>
@@ -1065,14 +1065,14 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB41"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="8.8984375" defaultRowHeight="13.8"/>
   <cols>
-    <col min="1" max="1" width="3.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.42578125" style="20" bestFit="1" customWidth="1"/>
-    <col min="3" max="16384" width="8.85546875" style="1"/>
+    <col min="1" max="1" width="3.3984375" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.3984375" style="20" bestFit="1" customWidth="1"/>
+    <col min="3" max="16384" width="8.8984375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="32.450000000000003" customHeight="1">
+    <row r="1" spans="1:28" ht="32.4" customHeight="1">
       <c r="A1" s="28" t="s">
         <v>31</v>
       </c>
@@ -1104,7 +1104,7 @@
       <c r="AA1" s="29"/>
       <c r="AB1" s="30"/>
     </row>
-    <row r="2" spans="1:28" ht="17.25">
+    <row r="2" spans="1:28" ht="16.8">
       <c r="A2" s="31" t="s">
         <v>32</v>
       </c>
@@ -1136,7 +1136,7 @@
       <c r="AA2" s="32"/>
       <c r="AB2" s="33"/>
     </row>
-    <row r="3" spans="1:28" ht="17.25">
+    <row r="3" spans="1:28" ht="16.8">
       <c r="A3" s="31" t="s">
         <v>33</v>
       </c>
@@ -1168,7 +1168,7 @@
       <c r="AA3" s="32"/>
       <c r="AB3" s="33"/>
     </row>
-    <row r="4" spans="1:28" ht="17.25">
+    <row r="4" spans="1:28" ht="16.8">
       <c r="A4" s="34" t="s">
         <v>0</v>
       </c>
@@ -1310,7 +1310,7 @@
       <c r="AA7" s="10"/>
       <c r="AB7" s="13"/>
     </row>
-    <row r="8" spans="1:28" ht="13.9" customHeight="1">
+    <row r="8" spans="1:28" ht="13.95" customHeight="1">
       <c r="A8" s="43" t="s">
         <v>8</v>
       </c>
@@ -1368,7 +1368,7 @@
       </c>
       <c r="AB8" s="47"/>
     </row>
-    <row r="9" spans="1:28" ht="30">
+    <row r="9" spans="1:28">
       <c r="A9" s="44"/>
       <c r="B9" s="15" t="s">
         <v>29</v>

</xml_diff>